<commit_message>
Update ESP32 PCB hardware files
</commit_message>
<xml_diff>
--- a/hardware/BOM.xlsx
+++ b/hardware/BOM.xlsx
@@ -73,28 +73,64 @@
     </r>
   </si>
   <si>
+    <t xml:space="preserve">100n</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1,C2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C_0603_1608Metric</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C14663</t>
+  </si>
+  <si>
     <t xml:space="preserve">10K</t>
   </si>
   <si>
-    <t xml:space="preserve">R2,R4,R1,R3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R_0805_2012Metric</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C17414</t>
+    <t xml:space="preserve">R1,R2,R3,R4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R_0603_1608Metric</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C101254</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CHANNELS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PinHeader_2x10_P2.54mm_Vertical</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5116480</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conn_01x15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J1,J2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PinSocket_1x15_P2.54mm_Vertical</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C7499333</t>
   </si>
   <si>
     <t xml:space="preserve">DEBUG</t>
   </si>
   <si>
-    <t xml:space="preserve">J5</t>
+    <t xml:space="preserve">J4</t>
   </si>
   <si>
     <t xml:space="preserve">PinHeader_1x03_P2.54mm_Vertical</t>
   </si>
   <si>
-    <t xml:space="preserve">C49257</t>
+    <t xml:space="preserve">C2937625</t>
   </si>
   <si>
     <t xml:space="preserve">SN74LVC245APW</t>
@@ -107,42 +143,6 @@
   </si>
   <si>
     <t xml:space="preserve">C7848</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Conn_01x15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">J1,J2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PinSocket_1x15_P2.54mm_Vertical</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C54104</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.1uF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C1,C2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C_0805_2012Metric</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C49678</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CHANNELS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">J6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PinHeader_2x10_P2.54mm_Vertical</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C5116480</t>
   </si>
 </sst>
 </file>

</xml_diff>